<commit_message>
Update Thai Emotion dataset file
</commit_message>
<xml_diff>
--- a/data/Thai Emotion.xlsx
+++ b/data/Thai Emotion.xlsx
@@ -351,7 +351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B712"/>
+  <dimension ref="A1:B780"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="38.5546875" customWidth="1" style="2" min="1" max="1"/>
@@ -7480,74 +7480,686 @@
         <v>3</v>
       </c>
     </row>
-    <row r="713" ht="16.5" customHeight="1" s="2"/>
-    <row r="714" ht="16.5" customHeight="1" s="2"/>
-    <row r="715" ht="16.5" customHeight="1" s="2"/>
-    <row r="716" ht="16.5" customHeight="1" s="2"/>
-    <row r="717" ht="16.5" customHeight="1" s="2"/>
-    <row r="718" ht="16.5" customHeight="1" s="2"/>
-    <row r="719" ht="16.5" customHeight="1" s="2"/>
-    <row r="720" ht="16.5" customHeight="1" s="2"/>
-    <row r="721" ht="16.5" customHeight="1" s="2"/>
-    <row r="722" ht="16.5" customHeight="1" s="2"/>
-    <row r="723" ht="16.5" customHeight="1" s="2"/>
-    <row r="724" ht="16.5" customHeight="1" s="2"/>
-    <row r="725" ht="16.5" customHeight="1" s="2"/>
-    <row r="726" ht="16.5" customHeight="1" s="2"/>
-    <row r="727" ht="16.5" customHeight="1" s="2"/>
-    <row r="728" ht="16.5" customHeight="1" s="2"/>
-    <row r="729" ht="16.5" customHeight="1" s="2"/>
-    <row r="730" ht="16.5" customHeight="1" s="2"/>
-    <row r="731" ht="16.5" customHeight="1" s="2"/>
-    <row r="732" ht="16.5" customHeight="1" s="2"/>
-    <row r="733" ht="16.5" customHeight="1" s="2"/>
-    <row r="734" ht="16.5" customHeight="1" s="2"/>
-    <row r="735" ht="16.5" customHeight="1" s="2"/>
-    <row r="736" ht="16.5" customHeight="1" s="2"/>
-    <row r="737" ht="16.5" customHeight="1" s="2"/>
-    <row r="738" ht="16.5" customHeight="1" s="2"/>
-    <row r="739" ht="16.5" customHeight="1" s="2"/>
-    <row r="740" ht="16.5" customHeight="1" s="2"/>
-    <row r="741" ht="16.5" customHeight="1" s="2"/>
-    <row r="742" ht="16.5" customHeight="1" s="2"/>
-    <row r="743" ht="16.5" customHeight="1" s="2"/>
-    <row r="744" ht="16.5" customHeight="1" s="2"/>
-    <row r="745" ht="16.5" customHeight="1" s="2"/>
-    <row r="746" ht="16.5" customHeight="1" s="2"/>
-    <row r="747" ht="16.5" customHeight="1" s="2"/>
-    <row r="748" ht="16.5" customHeight="1" s="2"/>
-    <row r="749" ht="16.5" customHeight="1" s="2"/>
-    <row r="750" ht="16.5" customHeight="1" s="2"/>
-    <row r="751" ht="16.5" customHeight="1" s="2"/>
-    <row r="752" ht="16.5" customHeight="1" s="2"/>
-    <row r="753" ht="16.5" customHeight="1" s="2"/>
-    <row r="754" ht="16.5" customHeight="1" s="2"/>
-    <row r="755" ht="16.5" customHeight="1" s="2"/>
-    <row r="756" ht="16.5" customHeight="1" s="2"/>
-    <row r="757" ht="16.5" customHeight="1" s="2"/>
-    <row r="758" ht="16.5" customHeight="1" s="2"/>
-    <row r="759" ht="16.5" customHeight="1" s="2"/>
-    <row r="760" ht="16.5" customHeight="1" s="2"/>
-    <row r="761" ht="16.5" customHeight="1" s="2"/>
-    <row r="762" ht="16.5" customHeight="1" s="2"/>
-    <row r="763" ht="16.5" customHeight="1" s="2"/>
-    <row r="764" ht="16.5" customHeight="1" s="2"/>
-    <row r="765" ht="16.5" customHeight="1" s="2"/>
-    <row r="766" ht="16.5" customHeight="1" s="2"/>
-    <row r="767" ht="16.5" customHeight="1" s="2"/>
-    <row r="768" ht="16.5" customHeight="1" s="2"/>
-    <row r="769" ht="16.5" customHeight="1" s="2"/>
-    <row r="770" ht="16.5" customHeight="1" s="2"/>
-    <row r="771" ht="16.5" customHeight="1" s="2"/>
-    <row r="772" ht="16.5" customHeight="1" s="2"/>
-    <row r="773" ht="16.5" customHeight="1" s="2"/>
-    <row r="774" ht="16.5" customHeight="1" s="2"/>
-    <row r="775" ht="16.5" customHeight="1" s="2"/>
-    <row r="776" ht="16.5" customHeight="1" s="2"/>
-    <row r="777" ht="16.5" customHeight="1" s="2"/>
-    <row r="778" ht="16.5" customHeight="1" s="2"/>
-    <row r="779" ht="16.5" customHeight="1" s="2"/>
-    <row r="780" ht="16.5" customHeight="1" s="2"/>
+    <row r="713" ht="16.5" customHeight="1" s="2">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>สั่งของไปนานแล้วยังไม่ได้ของเลย</t>
+        </is>
+      </c>
+      <c r="B713" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="714" ht="16.5" customHeight="1" s="2">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>สั่งของไปตั้งอาทิตย์แล้ว ยังไม่มาส่งเลย</t>
+        </is>
+      </c>
+      <c r="B714" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="715" ht="16.5" customHeight="1" s="2">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>รอของมาสองอาทิตย์แล้ว ทำไมยังไม่ส่ง</t>
+        </is>
+      </c>
+      <c r="B715" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="716" ht="16.5" customHeight="1" s="2">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>ส่งของช้าชิบหาย</t>
+        </is>
+      </c>
+      <c r="B716" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="717" ht="16.5" customHeight="1" s="2">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>ส่งของช้า แย่มาก</t>
+        </is>
+      </c>
+      <c r="B717" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="718" ht="16.5" customHeight="1" s="2">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>ค่าส่งแพงแถมส่งช้า</t>
+        </is>
+      </c>
+      <c r="B718" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="719" ht="16.5" customHeight="1" s="2">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>ขนส่งห่วยมาก</t>
+        </is>
+      </c>
+      <c r="B719" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="720" ht="16.5" customHeight="1" s="2">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>พัสดุหาย ขนส่งไม่รับผิดชอบเลย</t>
+        </is>
+      </c>
+      <c r="B720" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="721" ht="16.5" customHeight="1" s="2">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>ไรเดอร์ส่งผิดบ้าน หงุดหงิดมาก</t>
+        </is>
+      </c>
+      <c r="B721" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="722" ht="16.5" customHeight="1" s="2">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>บอกว่าจะส่งพรุ่งนี้ เลื่อนมาสามรอบแล้ว</t>
+        </is>
+      </c>
+      <c r="B722" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="723" ht="16.5" customHeight="1" s="2">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>เงินก็จ่ายแล้ว ของก็ยังไม่ได้</t>
+        </is>
+      </c>
+      <c r="B723" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="724" ht="16.5" customHeight="1" s="2">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>จ่ายเงินไปแล้วแต่ร้านไม่ส่งของ</t>
+        </is>
+      </c>
+      <c r="B724" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="725" ht="16.5" customHeight="1" s="2">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>ห่วยแตก</t>
+        </is>
+      </c>
+      <c r="B725" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="726" ht="16.5" customHeight="1" s="2">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>ห่วยมาก</t>
+        </is>
+      </c>
+      <c r="B726" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="727" ht="16.5" customHeight="1" s="2">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>ห่วยสุดๆ</t>
+        </is>
+      </c>
+      <c r="B727" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="728" ht="16.5" customHeight="1" s="2">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>ห่วยแตกจริงๆ</t>
+        </is>
+      </c>
+      <c r="B728" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="729" ht="16.5" customHeight="1" s="2">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>ห่วย!</t>
+        </is>
+      </c>
+      <c r="B729" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="730" ht="16.5" customHeight="1" s="2">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>บริการห่วยแตก</t>
+        </is>
+      </c>
+      <c r="B730" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="731" ht="16.5" customHeight="1" s="2">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>ร้านนี้ห่วยมาก ไม่ซื้ออีกแล้ว</t>
+        </is>
+      </c>
+      <c r="B731" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="732" ht="16.5" customHeight="1" s="2">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>แพงแล้วยังห่วยอีก</t>
+        </is>
+      </c>
+      <c r="B732" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="733" ht="16.5" customHeight="1" s="2">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>แอปค้างอีกแล้ว ห่วยจริงๆ</t>
+        </is>
+      </c>
+      <c r="B733" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="734" ht="16.5" customHeight="1" s="2">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>ห่วยจนไม่รู้จะพูดยังไง</t>
+        </is>
+      </c>
+      <c r="B734" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="735" ht="16.5" customHeight="1" s="2">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>ของไม่ตรงปก โกรธมาก</t>
+        </is>
+      </c>
+      <c r="B735" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="736" ht="16.5" customHeight="1" s="2">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>ของไม่ตรงปก ห่วยแตก</t>
+        </is>
+      </c>
+      <c r="B736" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="737" ht="16.5" customHeight="1" s="2">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>ได้ของผิดสี ไม่พอใจมาก</t>
+        </is>
+      </c>
+      <c r="B737" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="738" ht="16.5" customHeight="1" s="2">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>ได้ของไม่ครบ แย่มาก</t>
+        </is>
+      </c>
+      <c r="B738" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="739" ht="16.5" customHeight="1" s="2">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>ของพังตั้งแต่แกะกล่อง แย่มาก</t>
+        </is>
+      </c>
+      <c r="B739" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="740" ht="16.5" customHeight="1" s="2">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>สินค้าแย่มาก เสียเงินฟรี</t>
+        </is>
+      </c>
+      <c r="B740" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="741" ht="16.5" customHeight="1" s="2">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>แย่มาก ไม่แนะนำเลย</t>
+        </is>
+      </c>
+      <c r="B741" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="742" ht="16.5" customHeight="1" s="2">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>แย่ที่สุด ไม่ซื้ออีกแล้ว</t>
+        </is>
+      </c>
+      <c r="B742" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="743" ht="16.5" customHeight="1" s="2">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>แย่ที่สุด!</t>
+        </is>
+      </c>
+      <c r="B743" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="744" ht="16.5" customHeight="1" s="2">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>บริการแย่มาก!</t>
+        </is>
+      </c>
+      <c r="B744" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="745" ht="16.5" customHeight="1" s="2">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>ร้านนี้บริการแย่มาก</t>
+        </is>
+      </c>
+      <c r="B745" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="746" ht="16.5" customHeight="1" s="2">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>โทรหาร้านก็ไม่รับ ทักแชทก็ไม่ตอบ</t>
+        </is>
+      </c>
+      <c r="B746" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="747" ht="16.5" customHeight="1" s="2">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>ทักแชทไปหลายรอบ แอดมินไม่ตอบสักที</t>
+        </is>
+      </c>
+      <c r="B747" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="748" ht="16.5" customHeight="1" s="2">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>เรียกพนักงานตั้งนานไม่มีใครมา</t>
+        </is>
+      </c>
+      <c r="B748" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="749" ht="16.5" customHeight="1" s="2">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>รออาหารชั่วโมงนึงแล้วยังไม่ได้เลย</t>
+        </is>
+      </c>
+      <c r="B749" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="750" ht="16.5" customHeight="1" s="2">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>รอคิวตั้งนาน แล้วมาบอกว่าของหมด</t>
+        </is>
+      </c>
+      <c r="B750" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="751" ht="16.5" customHeight="1" s="2">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>สั่งข้าวไปตั้งนาน ได้มาเย็นชืด</t>
+        </is>
+      </c>
+      <c r="B751" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="752" ht="16.5" customHeight="1" s="2">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>อาหารไม่อร่อยแถมแพง ห่วยแตก</t>
+        </is>
+      </c>
+      <c r="B752" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="753" ht="16.5" customHeight="1" s="2">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>ขอคืนเงินแล้วไม่ยอมคืน โมโหมาก</t>
+        </is>
+      </c>
+      <c r="B753" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="754" ht="16.5" customHeight="1" s="2">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>โดนหลอกขายของปลอม</t>
+        </is>
+      </c>
+      <c r="B754" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="755" ht="16.5" customHeight="1" s="2">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>โกงตาชั่ง</t>
+        </is>
+      </c>
+      <c r="B755" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="756" ht="16.5" customHeight="1" s="2">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>ขายของเกินราคา</t>
+        </is>
+      </c>
+      <c r="B756" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="757" ht="16.5" customHeight="1" s="2">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>ไม่ซื่อสัตย์กับลูกค้าเลย</t>
+        </is>
+      </c>
+      <c r="B757" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="758" ht="16.5" customHeight="1" s="2">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>เสียเวลาชิบหาย</t>
+        </is>
+      </c>
+      <c r="B758" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="759" ht="16.5" customHeight="1" s="2">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>เสียเวลามาก ไม่พอใจเลย</t>
+        </is>
+      </c>
+      <c r="B759" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="760" ht="16.5" customHeight="1" s="2">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>ทำงานแบบนี้ได้ยังไง</t>
+        </is>
+      </c>
+      <c r="B760" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="761" ht="16.5" customHeight="1" s="2">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>ทำงานกันยังไงเนี่ย</t>
+        </is>
+      </c>
+      <c r="B761" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="762" ht="16.5" customHeight="1" s="2">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>มักง่ายมาก</t>
+        </is>
+      </c>
+      <c r="B762" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="763" ht="16.5" customHeight="1" s="2">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>ไม่มีความรับผิดชอบเลย</t>
+        </is>
+      </c>
+      <c r="B763" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="764" ht="16.5" customHeight="1" s="2">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>พูดจาไม่ดีใส่ลูกค้า แย่มาก</t>
+        </is>
+      </c>
+      <c r="B764" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="765" ht="16.5" customHeight="1" s="2">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>พนักงานหน้าบึ้งใส่ลูกค้า ไม่พอใจเลย</t>
+        </is>
+      </c>
+      <c r="B765" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="766" ht="16.5" customHeight="1" s="2">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>ร้านปิดก่อนเวลาไม่บอก เสียเที่ยวเลย</t>
+        </is>
+      </c>
+      <c r="B766" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="767" ht="16.5" customHeight="1" s="2">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>ส่งงานช้าแล้วยังมาโทษคนอื่น</t>
+        </is>
+      </c>
+      <c r="B767" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="768" ht="16.5" customHeight="1" s="2">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>ขับรถแย่มาก เกือบชนแล้ว</t>
+        </is>
+      </c>
+      <c r="B768" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="769" ht="16.5" customHeight="1" s="2">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>ไม่พอใจมาก!</t>
+        </is>
+      </c>
+      <c r="B769" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="770" ht="16.5" customHeight="1" s="2">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>โกรธมาก!</t>
+        </is>
+      </c>
+      <c r="B770" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="771" ht="16.5" customHeight="1" s="2">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>อย่ามาโกหก!</t>
+        </is>
+      </c>
+      <c r="B771" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="772" ht="16.5" customHeight="1" s="2">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>เย้! ได้ไปเที่ยวแล้ว</t>
+        </is>
+      </c>
+      <c r="B772" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="773" ht="16.5" customHeight="1" s="2">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>ดีใจมาก!</t>
+        </is>
+      </c>
+      <c r="B773" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="774" ht="16.5" customHeight="1" s="2">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>สุดยอด!</t>
+        </is>
+      </c>
+      <c r="B774" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="775" ht="16.5" customHeight="1" s="2">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>ได้ของแล้ว ดีใจจัง!</t>
+        </is>
+      </c>
+      <c r="B775" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="776" ht="16.5" customHeight="1" s="2">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>ของมาส่งไวมาก ประทับใจ</t>
+        </is>
+      </c>
+      <c r="B776" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="777" ht="16.5" customHeight="1" s="2">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>ร้านนี้บริการดีมาก</t>
+        </is>
+      </c>
+      <c r="B777" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="778" ht="16.5" customHeight="1" s="2">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>รักนะ!</t>
+        </is>
+      </c>
+      <c r="B778" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="779" ht="16.5" customHeight="1" s="2">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>คิดถึงมากๆ เลย!</t>
+        </is>
+      </c>
+      <c r="B779" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="780" ht="16.5" customHeight="1" s="2">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>แย่มาก สั่งของไปตั้งนานแล้วยังไม่ได้เลย ห่วยแตก!</t>
+        </is>
+      </c>
+      <c r="B780" t="n">
+        <v>3</v>
+      </c>
+    </row>
     <row r="781" ht="16.5" customHeight="1" s="2"/>
     <row r="782" ht="16.5" customHeight="1" s="2"/>
     <row r="783" ht="16.5" customHeight="1" s="2"/>

</xml_diff>